<commit_message>
Add Lecico; update Sidi Kerir; reposition to M&A/transaction CV (MOPCO analysis, MCDR, skills, engine, heading); 21 models
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/Sidi-Kerir-SKPC-Valuation-Model.xlsx
+++ b/models/Sidi-Kerir-SKPC-Valuation-Model.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7\SKPC - CA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed.wael\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998863F1-955A-4B52-A8F1-296F9316DC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F95069-673D-4DCF-B00B-5B140110E2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="1845" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FSM" sheetId="4" r:id="rId1"/>
     <sheet name="DCF" sheetId="2" r:id="rId2"/>
     <sheet name="WACC" sheetId="3" r:id="rId3"/>
+    <sheet name="Trading Comps" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="CIQWBGuid" localSheetId="1" hidden="1">"DCF_complete.xlsx"</definedName>
@@ -201,7 +202,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="315">
   <si>
     <t>Company Name</t>
   </si>
@@ -950,9 +951,6 @@
     <t>SKPC.CA</t>
   </si>
   <si>
-    <t>  Sidi Kerir Petrochemicals - SIDPEC</t>
-  </si>
-  <si>
     <t>Ethylene</t>
   </si>
   <si>
@@ -981,13 +979,181 @@
   </si>
   <si>
     <t>Plus: Net income</t>
+  </si>
+  <si>
+    <t>Comparable Companies Analysis (Trading Comps)</t>
+  </si>
+  <si>
+    <t>Refresh date:</t>
+  </si>
+  <si>
+    <t>GENERAL INFORMATION</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Misr Fertilizers (MOPCO)</t>
+  </si>
+  <si>
+    <t>Abu Qir Fertilizers</t>
+  </si>
+  <si>
+    <t>Exchange / Currency</t>
+  </si>
+  <si>
+    <t>EGX / EGP</t>
+  </si>
+  <si>
+    <t>Fiscal year end</t>
+  </si>
+  <si>
+    <t>Last closing price</t>
+  </si>
+  <si>
+    <t>Price as of</t>
+  </si>
+  <si>
+    <t>Basic shares outstanding</t>
+  </si>
+  <si>
+    <t>Options / RSUs / other dilution</t>
+  </si>
+  <si>
+    <t>Fully diluted shares</t>
+  </si>
+  <si>
+    <t>BALANCE SHEET DATA (latest reported)</t>
+  </si>
+  <si>
+    <t>Total debt (incl. leases)</t>
+  </si>
+  <si>
+    <t>Minority interest</t>
+  </si>
+  <si>
+    <t>Cash + liquid investments</t>
+  </si>
+  <si>
+    <t>Net debt / (net cash)</t>
+  </si>
+  <si>
+    <t>MARKET VALUATION</t>
+  </si>
+  <si>
+    <t>Market capitalization</t>
+  </si>
+  <si>
+    <t>Enterprise value (EV)</t>
+  </si>
+  <si>
+    <t>LTM FINANCIALS (millions, local currency)</t>
+  </si>
+  <si>
+    <t>LTM period</t>
+  </si>
+  <si>
+    <t>FY2025 (Dec-25)</t>
+  </si>
+  <si>
+    <t>EBITDA margin</t>
+  </si>
+  <si>
+    <t>TRADING MULTIPLES</t>
+  </si>
+  <si>
+    <t>EV / Revenue (LTM)</t>
+  </si>
+  <si>
+    <t>EV / EBITDA (LTM)</t>
+  </si>
+  <si>
+    <t>EV / EBIT (LTM)</t>
+  </si>
+  <si>
+    <t>P / E (LTM)</t>
+  </si>
+  <si>
+    <t>PEER STATISTICS (excl. MOPCO)</t>
+  </si>
+  <si>
+    <t>EV/Revenue</t>
+  </si>
+  <si>
+    <t>EV/EBITDA</t>
+  </si>
+  <si>
+    <t>EV/EBIT</t>
+  </si>
+  <si>
+    <t>P/E</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>Median</t>
+  </si>
+  <si>
+    <t>Via EV/EBITDA:</t>
+  </si>
+  <si>
+    <t>Peer median EV/EBITDA</t>
+  </si>
+  <si>
+    <t>x LTM EBITDA</t>
+  </si>
+  <si>
+    <t>Implied Enterprise Value</t>
+  </si>
+  <si>
+    <t>Less: net debt / plus net cash</t>
+  </si>
+  <si>
+    <t>Implied equity value</t>
+  </si>
+  <si>
+    <t>Implied value per share (EGP)</t>
+  </si>
+  <si>
+    <t>Via P/E:</t>
+  </si>
+  <si>
+    <t>Peer median P/E</t>
+  </si>
+  <si>
+    <t>Sidi Kerir Petrochemicals - SIDPEC</t>
+  </si>
+  <si>
+    <t>Egyptian Chemical Industries - KIMA</t>
+  </si>
+  <si>
+    <t>EGCH</t>
+  </si>
+  <si>
+    <t>MFPC</t>
+  </si>
+  <si>
+    <t>ABUK</t>
+  </si>
+  <si>
+    <t>Via (closest Egyptian peer):</t>
+  </si>
+  <si>
+    <t>IMPLIED VALUATION (from peer MEDIAN multiples)</t>
+  </si>
+  <si>
+    <t>x LTM net income</t>
+  </si>
+  <si>
+    <t>FULLY DILUTED SHARES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="33">
+  <numFmts count="35">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
@@ -1021,14 +1187,23 @@
     <numFmt numFmtId="193" formatCode="[$-409]mmmmm/yy;@"/>
     <numFmt numFmtId="194" formatCode="[$EGP]\ #,##0.00_);[Red]\([$EGP]\ #,##0.00\)"/>
     <numFmt numFmtId="195" formatCode="&quot;EGP&quot;\ #,##0.00"/>
+    <numFmt numFmtId="197" formatCode="#,##0;\(#,##0\)"/>
+    <numFmt numFmtId="198" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="44" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1309,6 +1484,19 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1336,7 +1524,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1615,495 +1803,530 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="37" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="193" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="37" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="193" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="279">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="174" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="175" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="18" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="173" fontId="19" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="174" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="175" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="5" applyBorder="1"/>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="5" applyBorder="1"/>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="3" applyBorder="1"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="180" fontId="22" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="180" fontId="26" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="37" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="180" fontId="22" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="25" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="25" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="8" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="181" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="180" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="177" fontId="19" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="182" fontId="19" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="181" fontId="19" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="172" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="22" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="184" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="183" fontId="28" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="37" fontId="19" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="37" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="187" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="188" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="188" fontId="5" fillId="0" borderId="9" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
+    <xf numFmtId="189" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="190" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="180" fontId="25" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="180" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="37" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="24" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="24" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyBorder="1"/>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="7" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="177" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="182" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="181" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="190" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="3" applyBorder="1"/>
+    <xf numFmtId="167" fontId="25" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="183" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="172" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="37" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="184" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="183" fontId="27" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="180" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="37" fontId="18" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="37" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="187" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="188" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="188" fontId="4" fillId="0" borderId="9" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="189" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="181" fontId="8" fillId="3" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="190" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="3" applyBorder="1"/>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="190" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="3" applyBorder="1"/>
-    <xf numFmtId="167" fontId="24" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="39" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="39" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="185" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="185" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="29" fillId="3" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="30" fillId="3" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="39" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="39" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="39" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="39" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="39" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="178" fontId="6" fillId="0" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="21" xfId="2" applyBorder="1"/>
-    <xf numFmtId="180" fontId="7" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="25" fillId="0" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="6" fillId="0" borderId="23" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="6" fillId="0" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="19" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="7" fillId="0" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="22" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="21" xfId="2" applyBorder="1"/>
+    <xf numFmtId="180" fontId="8" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="26" fillId="0" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="23" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="31" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="180" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="32" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="180" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="191" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="191" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="9" fontId="31" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="37" fontId="3" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="9" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="32" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="37" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="181" fontId="29" fillId="3" borderId="25" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="181" fontId="30" fillId="3" borderId="25" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="192" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="192" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="192" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="192" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="186" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="187" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="36" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="37" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="192" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="192" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="194" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="194" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="195" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="195" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="31" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="190" fontId="39" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="32" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="190" fontId="40" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="194" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="194" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="40" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="41" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="181" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="190" fontId="21" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="190" fontId="22" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="197" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="197" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="197" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="197" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="198" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="198" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="197" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="8">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 15" xfId="6" xr:uid="{6DDD7A4B-57F6-404C-BA97-B891B271587B}"/>
     <cellStyle name="Normal 2" xfId="3" xr:uid="{937EC6E3-AE83-4BBC-ACEF-6FAAD38BC45D}"/>
+    <cellStyle name="Normal 2 2" xfId="7" xr:uid="{69785CCC-C2BE-44A8-9900-2E031E0A4C9D}"/>
     <cellStyle name="Normal_DCF_Model" xfId="4" xr:uid="{EB47B55B-6DFA-4D8F-B164-61C0BEC4F72F}"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
@@ -2319,10 +2542,10 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>15.108175974374145</c:v>
+                  <c:v>15.111262233444371</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.253493818225028</c:v>
+                  <c:v>13.241776456306441</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>14.2</c:v>
@@ -2364,10 +2587,10 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>1.2095844364103847</c:v>
+                  <c:v>1.2150146703686637</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.85292341201861177</c:v>
+                  <c:v>0.85517652793150667</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5.740000000000002</c:v>
@@ -2434,10 +2657,10 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>16.31776041078453</c:v>
+                  <c:v>16.326276903813035</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14.10641723024364</c:v>
+                  <c:v>14.096952984237948</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>19.940000000000001</c:v>
@@ -2603,7 +2826,7 @@
                   <c:v>LTM EBITDA Purchase Multiple at 9.0%-11.0% Perpetuity Growth at 19.1% WACC</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>LTM EBITDA Purchase Multiple at 10.9x-11.9x Exit EBITDA Multiple at 19.1% WACC</c:v>
+                  <c:v>LTM EBITDA Purchase Multiple at 10.6x-11.6x Exit EBITDA Multiple at 19.1% WACC</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>LTM EBITDA Purchase Multiple at 17.1%-21.1% WACC at 8.4x Exit EBITDA</c:v>
@@ -2618,13 +2841,13 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>9.3586158704092597</c:v>
+                  <c:v>9.084787972969675</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.913986420007221</c:v>
+                  <c:v>10.608300252939573</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.8500712480062802</c:v>
+                  <c:v>9.5742073258227922</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2653,7 +2876,7 @@
                   <c:v>LTM EBITDA Purchase Multiple at 9.0%-11.0% Perpetuity Growth at 19.1% WACC</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>LTM EBITDA Purchase Multiple at 10.9x-11.9x Exit EBITDA Multiple at 19.1% WACC</c:v>
+                  <c:v>LTM EBITDA Purchase Multiple at 10.6x-11.6x Exit EBITDA Multiple at 19.1% WACC</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>LTM EBITDA Purchase Multiple at 17.1%-21.1% WACC at 8.4x Exit EBITDA</c:v>
@@ -2668,13 +2891,13 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.71527725207148407</c:v>
+                  <c:v>0.69691460495639035</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0143797434008981</c:v>
+                  <c:v>0.99015985747917412</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1601336911687188</c:v>
+                  <c:v>1.1229910454218572</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2724,7 +2947,7 @@
                   <c:v>LTM EBITDA Purchase Multiple at 9.0%-11.0% Perpetuity Growth at 19.1% WACC</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>LTM EBITDA Purchase Multiple at 10.9x-11.9x Exit EBITDA Multiple at 19.1% WACC</c:v>
+                  <c:v>LTM EBITDA Purchase Multiple at 10.6x-11.6x Exit EBITDA Multiple at 19.1% WACC</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>LTM EBITDA Purchase Multiple at 17.1%-21.1% WACC at 8.4x Exit EBITDA</c:v>
@@ -2739,13 +2962,13 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>10.073893122480744</c:v>
+                  <c:v>9.7817025779260653</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11.92836616340812</c:v>
+                  <c:v>11.598460110418747</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11.010204939174999</c:v>
+                  <c:v>10.697198371244649</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3094,7 +3317,7 @@
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="276" t="str">
         <f>Company_Name&amp;" - Financial Statement Model"</f>
-        <v>  Sidi Kerir Petrochemicals - SIDPEC - Financial Statement Model</v>
+        <v>Sidi Kerir Petrochemicals - SIDPEC - Financial Statement Model</v>
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -3121,7 +3344,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="275" t="s">
-        <v>249</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3137,7 +3360,7 @@
         <v>28</v>
       </c>
       <c r="D7" s="253">
-        <v>15.9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -6867,7 +7090,7 @@
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C155" s="16" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D155" s="267">
         <v>1136.896</v>
@@ -6901,7 +7124,7 @@
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C156" s="16" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D156" s="267">
         <v>8621.9889999999996</v>
@@ -6935,7 +7158,7 @@
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C157" s="16" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D157" s="267">
         <v>563.16300000000001</v>
@@ -6969,7 +7192,7 @@
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C158" s="16" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D158" s="267">
         <v>210.78700000000001</v>
@@ -7003,7 +7226,7 @@
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C159" s="16" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D159" s="267">
         <v>49.255000000000003</v>
@@ -7037,7 +7260,7 @@
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C160" s="16" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D160" s="267">
         <v>225.53700000000001</v>
@@ -7071,7 +7294,7 @@
     </row>
     <row r="161" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C161" s="16" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D161" s="267">
         <v>7.2859999999999996</v>
@@ -7105,7 +7328,7 @@
     </row>
     <row r="162" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C162" s="16" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D162" s="267">
         <v>46.491999999999997</v>
@@ -7139,7 +7362,7 @@
     </row>
     <row r="163" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C163" s="16" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D163" s="267">
         <v>2330.125</v>
@@ -7253,7 +7476,7 @@
     </row>
     <row r="168" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C168" s="16" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D168" s="6"/>
       <c r="E168" s="1">
@@ -7284,7 +7507,7 @@
     </row>
     <row r="169" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C169" s="16" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D169" s="6"/>
       <c r="E169" s="1">
@@ -7315,7 +7538,7 @@
     </row>
     <row r="170" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C170" s="16" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D170" s="6"/>
       <c r="E170" s="1">
@@ -7346,7 +7569,7 @@
     </row>
     <row r="171" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C171" s="16" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D171" s="6"/>
       <c r="E171" s="1">
@@ -7377,7 +7600,7 @@
     </row>
     <row r="172" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C172" s="16" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D172" s="6"/>
       <c r="E172" s="1">
@@ -7408,7 +7631,7 @@
     </row>
     <row r="173" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C173" s="16" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D173" s="6"/>
       <c r="E173" s="1">
@@ -7439,7 +7662,7 @@
     </row>
     <row r="174" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C174" s="16" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D174" s="6"/>
       <c r="E174" s="1">
@@ -7470,7 +7693,7 @@
     </row>
     <row r="175" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C175" s="16" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D175" s="6"/>
       <c r="E175" s="1">
@@ -7501,7 +7724,7 @@
     </row>
     <row r="176" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C176" s="16" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D176" s="6"/>
       <c r="E176" s="1">
@@ -8920,7 +9143,7 @@
     </row>
     <row r="231" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C231" s="16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D231" s="268">
         <f t="shared" ref="D231:K231" si="191">D33</f>
@@ -9127,7 +9350,7 @@
       </c>
       <c r="H4" s="55">
         <f>+WACC!E21</f>
-        <v>0.19090075624985225</v>
+        <v>0.19099252845010467</v>
       </c>
       <c r="I4" s="50" t="s">
         <v>49</v>
@@ -9146,7 +9369,8 @@
         <v>51</v>
       </c>
       <c r="H5" s="270">
-        <v>15.9</v>
+        <f>FSM!D7</f>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
@@ -9171,7 +9395,7 @@
       </c>
       <c r="C7" s="54"/>
       <c r="D7" s="54">
-        <v>46200</v>
+        <v>46210</v>
       </c>
       <c r="E7" s="58"/>
       <c r="F7" s="212" t="s">
@@ -9180,7 +9404,7 @@
       <c r="G7" s="58"/>
       <c r="H7" s="255">
         <f>C73</f>
-        <v>14.10641723024364</v>
+        <v>14.096952984237948</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
@@ -9190,14 +9414,14 @@
       <c r="C8" s="136"/>
       <c r="D8" s="136">
         <f>YEARFRAC(D7,D5)</f>
-        <v>0.51111111111111107</v>
+        <v>0.48333333333333334</v>
       </c>
       <c r="F8" s="212" t="s">
         <v>151</v>
       </c>
       <c r="H8" s="207">
         <f>H7/H5-1</f>
-        <v>-0.11280394778341896</v>
+        <v>-0.11894043848512825</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
@@ -9242,7 +9466,7 @@
       </c>
       <c r="C12" s="67">
         <f>D7</f>
-        <v>46200</v>
+        <v>46210</v>
       </c>
       <c r="D12" s="231">
         <f>D4</f>
@@ -9284,7 +9508,7 @@
       </c>
       <c r="C14" s="154">
         <f>E14*(1-$D$8)+D14*$D$8</f>
-        <v>14691863372.044445</v>
+        <v>14707731346.933334</v>
       </c>
       <c r="D14" s="176">
         <f>FSM!F16</f>
@@ -9344,7 +9568,7 @@
       </c>
       <c r="C16" s="154">
         <f>E16*(1-$D$8)+D16*$D$8</f>
-        <v>1352224115.0938244</v>
+        <v>1391519385.2696095</v>
       </c>
       <c r="D16" s="176">
         <f>FSM!F35</f>
@@ -9407,7 +9631,7 @@
       </c>
       <c r="C18" s="154">
         <f>E18*(1-$D$8)+D18*$D$8</f>
-        <v>1275292474.5924096</v>
+        <v>1314754923.2624326</v>
       </c>
       <c r="D18" s="176">
         <f>FSM!F24</f>
@@ -9797,7 +10021,7 @@
     <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" s="61" t="str">
         <f>"Present value of UFCF on "&amp;TEXT(D7,"mmm dd, yyyy")&amp;" valuation date"</f>
-        <v>Present value of UFCF on Jun 27, 2026 valuation date</v>
+        <v>Present value of UFCF on Jul 07, 2026 valuation date</v>
       </c>
       <c r="C35" s="62"/>
       <c r="D35" s="75"/>
@@ -9836,11 +10060,11 @@
       </c>
       <c r="D37" s="78">
         <f>D7</f>
-        <v>46200</v>
+        <v>46210</v>
       </c>
       <c r="E37" s="155">
         <f>IF($H$9=1,AVERAGE(E12,D37),E12)</f>
-        <v>46293.5</v>
+        <v>46298.5</v>
       </c>
       <c r="F37" s="155">
         <f>IF($H$9=1,AVERAGE(F12,E12),F12)</f>
@@ -9866,12 +10090,12 @@
       </c>
       <c r="C38" s="79">
         <f>D8</f>
-        <v>0.51111111111111107</v>
+        <v>0.48333333333333334</v>
       </c>
       <c r="D38" s="73"/>
       <c r="E38" s="80">
         <f>E30*C38</f>
-        <v>1167808626.0638523</v>
+        <v>1104340765.9516864</v>
       </c>
       <c r="F38" s="80">
         <f>F30</f>
@@ -9899,23 +10123,23 @@
       <c r="D39" s="72"/>
       <c r="E39" s="72">
         <f>E38/(1+$H$4)^((E37-$D$37)/365)</f>
-        <v>1116696255.780241</v>
+        <v>1058516817.2403573</v>
       </c>
       <c r="F39" s="72">
         <f t="shared" ref="F39:I39" si="11">F38/(1+$H$4)^((F37-$D$37)/365)</f>
-        <v>993024890.66048598</v>
+        <v>997713745.51085997</v>
       </c>
       <c r="G39" s="72">
         <f t="shared" si="11"/>
-        <v>923517471.75733399</v>
+        <v>927806531.38387656</v>
       </c>
       <c r="H39" s="72">
         <f t="shared" si="11"/>
-        <v>829648593.54519975</v>
+        <v>833437387.61072385</v>
       </c>
       <c r="I39" s="72">
         <f t="shared" si="11"/>
-        <v>744919660.61560857</v>
+        <v>748263857.11442149</v>
       </c>
       <c r="J39" s="68"/>
     </row>
@@ -9972,7 +10196,7 @@
       </c>
       <c r="C44" s="73">
         <f>C43/(H4-C42)</f>
-        <v>18179429081.881874</v>
+        <v>18161093881.897934</v>
       </c>
       <c r="E44" s="50" t="str">
         <f>"Terminal value in "&amp;YEAR(I12)</f>
@@ -9990,14 +10214,14 @@
       </c>
       <c r="C45" s="73">
         <f>C44/(1+H4)^((I37-D37)/365)</f>
-        <v>9014354340.7374172</v>
+        <v>9045690419.2655945</v>
       </c>
       <c r="E45" s="50" t="s">
         <v>84</v>
       </c>
       <c r="I45" s="73">
         <f>I44/(1+H4)^((I37-D37)/365)</f>
-        <v>11522017507.470791</v>
+        <v>11573743744.063742</v>
       </c>
       <c r="J45" s="73"/>
     </row>
@@ -10007,14 +10231,14 @@
       </c>
       <c r="C46" s="68">
         <f>SUM(E39:I39)</f>
-        <v>4607806872.3588696</v>
+        <v>4565738338.860239</v>
       </c>
       <c r="E46" s="50" t="s">
         <v>85</v>
       </c>
       <c r="I46" s="73">
         <f>C46</f>
-        <v>4607806872.3588696</v>
+        <v>4565738338.860239</v>
       </c>
       <c r="J46" s="73"/>
     </row>
@@ -10024,14 +10248,14 @@
       </c>
       <c r="C47" s="85">
         <f>C45+C46</f>
-        <v>13622161213.096287</v>
+        <v>13611428758.125834</v>
       </c>
       <c r="E47" s="71" t="s">
         <v>87</v>
       </c>
       <c r="I47" s="85">
         <f>I45+I46</f>
-        <v>16129824379.82966</v>
+        <v>16139482082.923981</v>
       </c>
       <c r="J47" s="85"/>
     </row>
@@ -10041,14 +10265,14 @@
       </c>
       <c r="C49" s="87">
         <f>C45/C47</f>
-        <v>0.66174186310987537</v>
+        <v>0.6645658277324813</v>
       </c>
       <c r="E49" s="86" t="s">
         <v>88</v>
       </c>
       <c r="I49" s="87">
         <f>I45/I47</f>
-        <v>0.71433000360990107</v>
+        <v>0.7171075059657015</v>
       </c>
       <c r="J49" s="87"/>
     </row>
@@ -10058,7 +10282,7 @@
       </c>
       <c r="C50" s="87">
         <f>1-C49</f>
-        <v>0.33825813689012463</v>
+        <v>0.3354341722675187</v>
       </c>
       <c r="E50" s="86" t="s">
         <v>90</v>
@@ -10066,7 +10290,7 @@
       <c r="G50" s="88"/>
       <c r="I50" s="89">
         <f>1-I49</f>
-        <v>0.28566999639009893</v>
+        <v>0.2828924940342985</v>
       </c>
       <c r="J50" s="89"/>
     </row>
@@ -10076,14 +10300,14 @@
       </c>
       <c r="C51" s="90">
         <f>C47/I16</f>
-        <v>4.9243754356585656</v>
+        <v>4.9204956814261758</v>
       </c>
       <c r="E51" s="50" t="s">
         <v>92</v>
       </c>
       <c r="I51" s="217">
         <f>(H4-I38/I44)/(1+I38/I44)</f>
-        <v>0.11858234660800193</v>
+        <v>0.1186685458673214</v>
       </c>
       <c r="J51" s="91"/>
     </row>
@@ -10277,11 +10501,11 @@
       </c>
       <c r="C69" s="108">
         <f>C47</f>
-        <v>13622161213.096287</v>
+        <v>13611428758.125834</v>
       </c>
       <c r="D69" s="108">
         <f>I47</f>
-        <v>16129824379.82966</v>
+        <v>16139482082.923981</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.25">
@@ -10303,11 +10527,11 @@
       </c>
       <c r="C71" s="110">
         <f>C69-C70</f>
-        <v>15996677139.096287</v>
+        <v>15985944684.125834</v>
       </c>
       <c r="D71" s="110">
         <f t="shared" ref="D71" si="13">D69-D70</f>
-        <v>18504340305.829659</v>
+        <v>18513998008.923981</v>
       </c>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.25">
@@ -10329,11 +10553,11 @@
       </c>
       <c r="C73" s="254">
         <f>C71/C72</f>
-        <v>14.10641723024364</v>
+        <v>14.096952984237948</v>
       </c>
       <c r="D73" s="254">
         <f t="shared" ref="D73" si="15">D71/D72</f>
-        <v>16.31776041078453</v>
+        <v>16.326276903813035</v>
       </c>
     </row>
     <row r="75" spans="2:6" ht="17.25" x14ac:dyDescent="0.4">
@@ -10357,11 +10581,11 @@
       </c>
       <c r="C77" s="236">
         <f>C69/$C$14</f>
-        <v>0.92719084490102333</v>
+        <v>0.92546079589384889</v>
       </c>
       <c r="D77" s="236">
         <f>D69/$C$14</f>
-        <v>1.0978746515245545</v>
+        <v>1.0973468104779585</v>
       </c>
     </row>
     <row r="78" spans="2:6" x14ac:dyDescent="0.25">
@@ -10370,11 +10594,11 @@
       </c>
       <c r="C78" s="237">
         <f>C69/$C$16</f>
-        <v>10.073893122480744</v>
+        <v>9.7817025779260653</v>
       </c>
       <c r="D78" s="237">
         <f>D69/$C$16</f>
-        <v>11.92836616340812</v>
+        <v>11.598460110418747</v>
       </c>
     </row>
     <row r="79" spans="2:6" x14ac:dyDescent="0.25">
@@ -10383,11 +10607,11 @@
       </c>
       <c r="C79" s="237">
         <f>C69/$C$18</f>
-        <v>10.681597738942202</v>
+        <v>10.352825851642706</v>
       </c>
       <c r="D79" s="237">
         <f>D69/$C$18</f>
-        <v>12.647941316351639</v>
+        <v>12.275658221439075</v>
       </c>
     </row>
     <row r="80" spans="2:6" ht="17.25" x14ac:dyDescent="0.4">
@@ -10416,11 +10640,11 @@
       </c>
       <c r="C82" s="236">
         <f>C69/$E$14</f>
-        <v>0.90912386730209771</v>
+        <v>0.90840759836240814</v>
       </c>
       <c r="D82" s="236">
         <f>D69/$E$14</f>
-        <v>1.0764817777223548</v>
+        <v>1.0771263192344551</v>
       </c>
       <c r="E82" s="111"/>
       <c r="F82" s="111"/>
@@ -10431,11 +10655,11 @@
       </c>
       <c r="C83" s="237">
         <f>C69/$E$16</f>
-        <v>6.5640836997202046</v>
+        <v>6.5589120730137314</v>
       </c>
       <c r="D83" s="237">
         <f>D69/$E$16</f>
-        <v>7.7724463566911286</v>
+        <v>7.7771000948510629</v>
       </c>
       <c r="E83" s="111"/>
       <c r="F83" s="111"/>
@@ -10446,11 +10670,11 @@
       </c>
       <c r="C84" s="237">
         <f>C69/$E$18</f>
-        <v>6.8063109816218788</v>
+        <v>6.8009485119680226</v>
       </c>
       <c r="D84" s="237">
         <f>D69/$E$18</f>
-        <v>8.059264538913288</v>
+        <v>8.0640900089396546</v>
       </c>
       <c r="E84" s="111"/>
       <c r="F84" s="111"/>
@@ -10524,7 +10748,7 @@
       <c r="C90" s="117"/>
       <c r="D90" s="159">
         <f>C73</f>
-        <v>14.10641723024364</v>
+        <v>14.096952984237948</v>
       </c>
       <c r="E90" s="194">
         <f>F90-0.005</f>
@@ -10549,7 +10773,7 @@
       <c r="K90" s="122"/>
       <c r="L90" s="119">
         <f>C78</f>
-        <v>10.073893122480744</v>
+        <v>9.7817025779260653</v>
       </c>
       <c r="M90" s="194">
         <f>N90-0.005</f>
@@ -10576,86 +10800,86 @@
       <c r="B91" s="112"/>
       <c r="D91" s="192">
         <f>D92+0.01</f>
-        <v>0.21090075624985227</v>
+        <v>0.21099252845010469</v>
       </c>
       <c r="E91" s="120">
         <f t="dataTable" ref="E91:I95" dt2D="1" dtr="1" r1="C42" r2="H4" ca="1"/>
-        <v>11.572514533131713</v>
+        <v>11.559878109408059</v>
       </c>
       <c r="F91" s="120">
-        <v>11.328128336193004</v>
+        <v>11.314627950228195</v>
       </c>
       <c r="G91" s="120">
-        <v>11.328128336193004</v>
+        <v>11.314627950228195</v>
       </c>
       <c r="H91" s="120">
-        <v>11.572514533131713</v>
+        <v>11.559878109408059</v>
       </c>
       <c r="I91" s="120">
-        <v>12.127396358144505</v>
+        <v>12.116666716521417</v>
       </c>
       <c r="J91" s="121"/>
       <c r="L91" s="192">
         <f>L92+0.01</f>
-        <v>0.21090075624985227</v>
+        <v>0.21099252845010469</v>
       </c>
       <c r="M91" s="122">
         <f t="dataTable" ref="M91:Q95" dt2D="1" dtr="1" r1="C42" r2="H4" ca="1"/>
-        <v>7.9489157415489213</v>
+        <v>7.7141475452668109</v>
       </c>
       <c r="N91" s="122">
-        <v>7.743968984398931</v>
+        <v>7.5142842279073614</v>
       </c>
       <c r="O91" s="122">
-        <v>7.743968984398931</v>
+        <v>7.5142842279073614</v>
       </c>
       <c r="P91" s="122">
-        <v>7.9489157415489213</v>
+        <v>7.7141475452668109</v>
       </c>
       <c r="Q91" s="122">
-        <v>8.4142498400469705</v>
+        <v>8.1678949289902594</v>
       </c>
     </row>
     <row r="92" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="112"/>
       <c r="D92" s="192">
         <f>D93+0.01</f>
-        <v>0.20090075624985226</v>
+        <v>0.20099252845010468</v>
       </c>
       <c r="E92" s="120">
-        <v>12.337464402691671</v>
+        <v>12.32529850364824</v>
       </c>
       <c r="F92" s="120">
-        <v>12.040727324309374</v>
+        <v>12.027619668227269</v>
       </c>
       <c r="G92" s="120">
-        <v>12.040727324309374</v>
+        <v>12.027619668227269</v>
       </c>
       <c r="H92" s="120">
-        <v>12.337464402691671</v>
+        <v>12.32529850364824</v>
       </c>
       <c r="I92" s="120">
-        <v>13.019164977991979</v>
+        <v>13.009082171934548</v>
       </c>
       <c r="J92" s="121"/>
       <c r="L92" s="192">
         <f>L93+0.01</f>
-        <v>0.20090075624985226</v>
+        <v>0.20099252845010468</v>
       </c>
       <c r="M92" s="122">
-        <v>8.5904167637524829</v>
+        <v>8.337916596748757</v>
       </c>
       <c r="N92" s="122">
-        <v>8.3415675950906909</v>
+        <v>8.0953272351194343</v>
       </c>
       <c r="O92" s="122">
-        <v>8.3415675950906909</v>
+        <v>8.0953272351194343</v>
       </c>
       <c r="P92" s="122">
-        <v>8.5904167637524829</v>
+        <v>8.337916596748757</v>
       </c>
       <c r="Q92" s="122">
-        <v>9.1621033974706734</v>
+        <v>8.8951568968444938</v>
       </c>
     </row>
     <row r="93" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10665,22 +10889,22 @@
       </c>
       <c r="D93" s="123">
         <f>WACC!$E$21</f>
-        <v>0.19090075624985225</v>
+        <v>0.19099252845010467</v>
       </c>
       <c r="E93" s="120">
-        <v>13.253493818225028</v>
+        <v>13.241776456306441</v>
       </c>
       <c r="F93" s="120">
-        <v>12.887437021648543</v>
+        <v>12.874700230814282</v>
       </c>
       <c r="G93" s="120">
-        <v>12.887437021648543</v>
+        <v>12.874700230814282</v>
       </c>
       <c r="H93" s="120">
-        <v>13.253493818225028</v>
+        <v>13.241776456306441</v>
       </c>
       <c r="I93" s="120">
-        <v>14.10641723024364</v>
+        <v>14.096952984237948</v>
       </c>
       <c r="J93" s="121"/>
       <c r="K93" s="117" t="s">
@@ -10688,64 +10912,64 @@
       </c>
       <c r="L93" s="123">
         <f>WACC!$E$21</f>
-        <v>0.19090075624985225</v>
+        <v>0.19099252845010467</v>
       </c>
       <c r="M93" s="122">
-        <v>9.3586158704092597</v>
+        <v>9.084787972969675</v>
       </c>
       <c r="N93" s="122">
-        <v>9.0516339118091995</v>
+        <v>8.7856441420503124</v>
       </c>
       <c r="O93" s="122">
-        <v>9.0516339118091995</v>
+        <v>8.7856441420503124</v>
       </c>
       <c r="P93" s="122">
-        <v>9.3586158704092597</v>
+        <v>9.084787972969675</v>
       </c>
       <c r="Q93" s="122">
-        <v>10.073893122480744</v>
+        <v>9.7817025779260653</v>
       </c>
     </row>
     <row r="94" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="112"/>
       <c r="D94" s="192">
         <f t="shared" ref="D94:D95" si="16">D93-0.01</f>
-        <v>0.18090075624985225</v>
+        <v>0.18099252845010466</v>
       </c>
       <c r="E94" s="120">
-        <v>14.370449451558313</v>
+        <v>14.359101644360823</v>
       </c>
       <c r="F94" s="120">
-        <v>13.910199105593559</v>
+        <v>13.897764837821294</v>
       </c>
       <c r="G94" s="120">
-        <v>13.910199105593559</v>
+        <v>13.897764837821294</v>
       </c>
       <c r="H94" s="120">
-        <v>14.370449451558313</v>
+        <v>14.359101644360823</v>
       </c>
       <c r="I94" s="120">
-        <v>15.461622347543615</v>
+        <v>15.452656503661403</v>
       </c>
       <c r="J94" s="121"/>
       <c r="L94" s="192">
         <f t="shared" ref="L94:L95" si="17">L93-0.01</f>
-        <v>0.18090075624985225</v>
+        <v>0.18099252845010466</v>
       </c>
       <c r="M94" s="122">
-        <v>10.295315396812883</v>
+        <v>9.9953371012580874</v>
       </c>
       <c r="N94" s="122">
-        <v>9.9093409961952634</v>
+        <v>9.6193768780992386</v>
       </c>
       <c r="O94" s="122">
-        <v>9.9093409961952634</v>
+        <v>9.6193768780992386</v>
       </c>
       <c r="P94" s="122">
-        <v>10.295315396812883</v>
+        <v>9.9953371012580874</v>
       </c>
       <c r="Q94" s="122">
-        <v>11.210393045728704</v>
+        <v>10.886514919960616</v>
       </c>
     </row>
     <row r="95" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10754,42 +10978,42 @@
       </c>
       <c r="D95" s="193">
         <f t="shared" si="16"/>
-        <v>0.17090075624985224</v>
+        <v>0.17099252845010465</v>
       </c>
       <c r="E95" s="120">
-        <v>15.762823196967117</v>
+        <v>15.751652915622039</v>
       </c>
       <c r="F95" s="120">
-        <v>15.17048508240037</v>
+        <v>15.158196073891446</v>
       </c>
       <c r="G95" s="120">
-        <v>15.17048508240037</v>
+        <v>15.158196073891446</v>
       </c>
       <c r="H95" s="120">
-        <v>15.762823196967117</v>
+        <v>15.751652915622039</v>
       </c>
       <c r="I95" s="120">
-        <v>17.198133472575105</v>
+        <v>17.189349401733089</v>
       </c>
       <c r="J95" s="121"/>
       <c r="L95" s="193">
         <f t="shared" si="17"/>
-        <v>0.17090075624985224</v>
+        <v>0.17099252845010465</v>
       </c>
       <c r="M95" s="122">
-        <v>11.462985614840335</v>
+        <v>11.130178022862822</v>
       </c>
       <c r="N95" s="122">
-        <v>10.966239983387014</v>
+        <v>10.646548354712637</v>
       </c>
       <c r="O95" s="122">
-        <v>10.966239983387014</v>
+        <v>10.646548354712637</v>
       </c>
       <c r="P95" s="122">
-        <v>11.462985614840335</v>
+        <v>11.130178022862822</v>
       </c>
       <c r="Q95" s="122">
-        <v>12.666663196367955</v>
+        <v>12.301809429876277</v>
       </c>
     </row>
     <row r="96" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10845,7 +11069,7 @@
       <c r="B99" s="112"/>
       <c r="D99" s="160">
         <f>D73</f>
-        <v>16.31776041078453</v>
+        <v>16.326276903813035</v>
       </c>
       <c r="E99" s="161">
         <f>+F99-0.5</f>
@@ -10870,7 +11094,7 @@
       <c r="J99" s="219"/>
       <c r="L99" s="119">
         <f>D78</f>
-        <v>11.92836616340812</v>
+        <v>11.598460110418747</v>
       </c>
       <c r="M99" s="161">
         <f>+N99-0.5</f>
@@ -10897,86 +11121,86 @@
       <c r="B100" s="112"/>
       <c r="D100" s="192">
         <f>D101+0.01</f>
-        <v>0.21090075624985227</v>
+        <v>0.21099252845010469</v>
       </c>
       <c r="E100" s="120">
         <f t="dataTable" ref="E100:I104" dt2D="1" dtr="1" r1="I43" r2="H4" ca="1"/>
-        <v>14.405196423262726</v>
+        <v>14.410812256169216</v>
       </c>
       <c r="F100" s="120">
-        <v>13.839523635755215</v>
+        <v>13.842337758794288</v>
       </c>
       <c r="G100" s="120">
-        <v>13.839523635755215</v>
+        <v>13.842337758794288</v>
       </c>
       <c r="H100" s="120">
-        <v>14.405196423262726</v>
+        <v>14.410812256169216</v>
       </c>
       <c r="I100" s="120">
-        <v>15.536541998277745</v>
+        <v>15.547761250919066</v>
       </c>
       <c r="J100" s="121"/>
       <c r="L100" s="192">
         <f>L101+0.01</f>
-        <v>0.21090075624985227</v>
+        <v>0.21099252845010469</v>
       </c>
       <c r="M100" s="122">
         <f t="dataTable" ref="M100:Q104" dt2D="1" dtr="1" r1="I43" r2="H4" ca="1"/>
-        <v>10.324454846015851</v>
+        <v>10.037477968580143</v>
       </c>
       <c r="N100" s="122">
-        <v>9.8500712480062802</v>
+        <v>9.5742073258227922</v>
       </c>
       <c r="O100" s="122">
-        <v>9.8500712480062802</v>
+        <v>9.5742073258227922</v>
       </c>
       <c r="P100" s="122">
-        <v>10.324454846015851</v>
+        <v>10.037477968580143</v>
       </c>
       <c r="Q100" s="122">
-        <v>11.273222042034991</v>
+        <v>10.964019254094845</v>
       </c>
     </row>
     <row r="101" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="112"/>
       <c r="D101" s="192">
         <f>D102+0.01</f>
-        <v>0.20090075624985226</v>
+        <v>0.20099252845010468</v>
       </c>
       <c r="E101" s="120">
-        <v>14.749658455951906</v>
+        <v>14.754069535546472</v>
       </c>
       <c r="F101" s="120">
-        <v>14.164834325864298</v>
+        <v>14.166483831701733</v>
       </c>
       <c r="G101" s="120">
-        <v>14.164834325864298</v>
+        <v>14.166483831701733</v>
       </c>
       <c r="H101" s="120">
-        <v>14.749658455951906</v>
+        <v>14.754069535546472</v>
       </c>
       <c r="I101" s="120">
-        <v>15.919306716127116</v>
+        <v>15.929240943235952</v>
       </c>
       <c r="J101" s="121"/>
       <c r="L101" s="192">
         <f>L102+0.01</f>
-        <v>0.20090075624985226</v>
+        <v>0.20099252845010468</v>
       </c>
       <c r="M101" s="122">
-        <v>10.613327038657104</v>
+        <v>10.317210869849349</v>
       </c>
       <c r="N101" s="122">
-        <v>10.122882772712821</v>
+        <v>9.8383658065225212</v>
       </c>
       <c r="O101" s="122">
-        <v>10.122882772712821</v>
+        <v>9.8383658065225212</v>
       </c>
       <c r="P101" s="122">
-        <v>10.613327038657104</v>
+        <v>10.317210869849349</v>
       </c>
       <c r="Q101" s="122">
-        <v>11.594215570545664</v>
+        <v>11.274900996503007</v>
       </c>
     </row>
     <row r="102" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10986,22 +11210,22 @@
       </c>
       <c r="D102" s="123">
         <f>WACC!$E$21</f>
-        <v>0.19090075624985225</v>
+        <v>0.19099252845010467</v>
       </c>
       <c r="E102" s="120">
-        <v>15.108175974374145</v>
+        <v>15.111262233444371</v>
       </c>
       <c r="F102" s="120">
-        <v>14.503383756168951</v>
+        <v>14.503754898260039</v>
       </c>
       <c r="G102" s="120">
-        <v>14.503383756168951</v>
+        <v>14.503754898260039</v>
       </c>
       <c r="H102" s="120">
-        <v>15.108175974374145</v>
+        <v>15.111262233444371</v>
       </c>
       <c r="I102" s="120">
-        <v>16.31776041078453</v>
+        <v>16.326276903813035</v>
       </c>
       <c r="J102" s="121"/>
       <c r="K102" s="117" t="s">
@@ -11009,106 +11233,106 @@
       </c>
       <c r="L102" s="123">
         <f>WACC!$E$21</f>
-        <v>0.19090075624985225</v>
+        <v>0.19099252845010467</v>
       </c>
       <c r="M102" s="122">
-        <v>10.913986420007221</v>
+        <v>10.608300252939573</v>
       </c>
       <c r="N102" s="122">
-        <v>10.406796548306772</v>
+        <v>10.113220324199986</v>
       </c>
       <c r="O102" s="122">
-        <v>10.406796548306772</v>
+        <v>10.113220324199986</v>
       </c>
       <c r="P102" s="122">
-        <v>10.913986420007221</v>
+        <v>10.608300252939573</v>
       </c>
       <c r="Q102" s="122">
-        <v>11.92836616340812</v>
+        <v>11.598460110418747</v>
       </c>
     </row>
     <row r="103" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="112"/>
       <c r="D103" s="192">
         <f t="shared" ref="D103:D104" si="18">D102-0.01</f>
-        <v>0.18090075624985225</v>
+        <v>0.18099252845010466</v>
       </c>
       <c r="E103" s="120">
-        <v>15.48145903849635</v>
+        <v>15.483091168284176</v>
       </c>
       <c r="F103" s="120">
-        <v>14.855839852031218</v>
+        <v>14.854810166882253</v>
       </c>
       <c r="G103" s="120">
-        <v>14.855839852031218</v>
+        <v>14.854810166882253</v>
       </c>
       <c r="H103" s="120">
-        <v>15.48145903849635</v>
+        <v>15.483091168284176</v>
       </c>
       <c r="I103" s="120">
-        <v>16.73269741142661</v>
+        <v>16.739653171088023</v>
       </c>
       <c r="J103" s="121"/>
       <c r="L103" s="192">
         <f t="shared" ref="L103:L104" si="19">L102-0.01</f>
-        <v>0.18090075624985225</v>
+        <v>0.18099252845010466</v>
       </c>
       <c r="M103" s="122">
-        <v>11.227028459407036</v>
+        <v>10.911317240393645</v>
       </c>
       <c r="N103" s="122">
-        <v>10.702372709274792</v>
+        <v>10.399308091881682</v>
       </c>
       <c r="O103" s="122">
-        <v>10.702372709274792</v>
+        <v>10.399308091881682</v>
       </c>
       <c r="P103" s="122">
-        <v>11.227028459407036</v>
+        <v>10.911317240393645</v>
       </c>
       <c r="Q103" s="122">
-        <v>12.276339959671521</v>
+        <v>11.935335537417567</v>
       </c>
     </row>
     <row r="104" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="112"/>
       <c r="D104" s="193">
         <f t="shared" si="18"/>
-        <v>0.17090075624985224</v>
+        <v>0.17099252845010465</v>
       </c>
       <c r="E104" s="120">
-        <v>15.870260270363787</v>
+        <v>15.870298999765009</v>
       </c>
       <c r="F104" s="120">
-        <v>15.222910543983746</v>
+        <v>15.220348172540938</v>
       </c>
       <c r="G104" s="120">
-        <v>15.222910543983746</v>
+        <v>15.220348172540938</v>
       </c>
       <c r="H104" s="120">
-        <v>15.870260270363787</v>
+        <v>15.870298999765009</v>
       </c>
       <c r="I104" s="120">
-        <v>17.164959723123868</v>
+        <v>17.170200654213147</v>
       </c>
       <c r="J104" s="121"/>
       <c r="L104" s="193">
         <f t="shared" si="19"/>
-        <v>0.17090075624985224</v>
+        <v>0.17099252845010465</v>
       </c>
       <c r="M104" s="122">
-        <v>11.553084319538682</v>
+        <v>11.226867052740808</v>
       </c>
       <c r="N104" s="122">
-        <v>11.010204939174999</v>
+        <v>10.697198371244649</v>
       </c>
       <c r="O104" s="122">
-        <v>11.010204939174999</v>
+        <v>10.697198371244649</v>
       </c>
       <c r="P104" s="122">
-        <v>11.553084319538682</v>
+        <v>11.226867052740808</v>
       </c>
       <c r="Q104" s="122">
-        <v>12.638843080266049</v>
+        <v>12.286204415733117</v>
       </c>
     </row>
     <row r="105" spans="2:17" x14ac:dyDescent="0.25">
@@ -11231,15 +11455,15 @@
       </c>
       <c r="C128" s="163">
         <f>E102</f>
-        <v>15.108175974374145</v>
+        <v>15.111262233444371</v>
       </c>
       <c r="D128" s="163">
         <f>E128-C128</f>
-        <v>1.2095844364103847</v>
+        <v>1.2150146703686637</v>
       </c>
       <c r="E128" s="164">
         <f>I102</f>
-        <v>16.31776041078453</v>
+        <v>16.326276903813035</v>
       </c>
       <c r="G128" s="162" t="str">
         <f>"LTM EBITDA Purchase Multiple at "&amp;TEXT(M90,"0.0%")&amp;"-"&amp;TEXT(Q90,"0.0%")&amp;" Perpetuity Growth at "&amp;TEXT(L93,"0.0%")&amp;" WACC"</f>
@@ -11254,15 +11478,15 @@
       <c r="N128"/>
       <c r="O128" s="171">
         <f>M93</f>
-        <v>9.3586158704092597</v>
+        <v>9.084787972969675</v>
       </c>
       <c r="P128" s="171">
         <f>Q128-O128</f>
-        <v>0.71527725207148407</v>
+        <v>0.69691460495639035</v>
       </c>
       <c r="Q128" s="172">
         <f>Q93</f>
-        <v>10.073893122480744</v>
+        <v>9.7817025779260653</v>
       </c>
     </row>
     <row r="129" spans="2:17" x14ac:dyDescent="0.25">
@@ -11272,19 +11496,19 @@
       </c>
       <c r="C129" s="163">
         <f>E93</f>
-        <v>13.253493818225028</v>
+        <v>13.241776456306441</v>
       </c>
       <c r="D129" s="163">
         <f>E129-C129</f>
-        <v>0.85292341201861177</v>
+        <v>0.85517652793150667</v>
       </c>
       <c r="E129" s="164">
         <f>I93</f>
-        <v>14.10641723024364</v>
+        <v>14.096952984237948</v>
       </c>
       <c r="G129" s="165" t="str">
         <f>"LTM EBITDA Purchase Multiple at "&amp;TEXT(M102,"0.0x")&amp;"-"&amp;TEXT(Q102,"0.0x")&amp;" Exit EBITDA Multiple at "&amp;TEXT(L102,"0.0%")&amp;" WACC"</f>
-        <v>LTM EBITDA Purchase Multiple at 10.9x-11.9x Exit EBITDA Multiple at 19.1% WACC</v>
+        <v>LTM EBITDA Purchase Multiple at 10.6x-11.6x Exit EBITDA Multiple at 19.1% WACC</v>
       </c>
       <c r="H129"/>
       <c r="I129"/>
@@ -11295,15 +11519,15 @@
       <c r="N129"/>
       <c r="O129" s="171">
         <f>M102</f>
-        <v>10.913986420007221</v>
+        <v>10.608300252939573</v>
       </c>
       <c r="P129" s="171">
         <f>Q129-O129</f>
-        <v>1.0143797434008981</v>
+        <v>0.99015985747917412</v>
       </c>
       <c r="Q129" s="172">
         <f>Q102</f>
-        <v>11.92836616340812</v>
+        <v>11.598460110418747</v>
       </c>
     </row>
     <row r="130" spans="2:17" x14ac:dyDescent="0.25">
@@ -11333,15 +11557,15 @@
       <c r="N130" s="39"/>
       <c r="O130" s="168">
         <f>O100</f>
-        <v>9.8500712480062802</v>
+        <v>9.5742073258227922</v>
       </c>
       <c r="P130" s="168">
         <f>Q130-O130</f>
-        <v>1.1601336911687188</v>
+        <v>1.1229910454218572</v>
       </c>
       <c r="Q130" s="174">
         <f>O104</f>
-        <v>11.010204939174999</v>
+        <v>10.697198371244649</v>
       </c>
     </row>
     <row r="131" spans="2:17" x14ac:dyDescent="0.25">
@@ -11514,12 +11738,12 @@
       </c>
       <c r="C18" s="69">
         <f>DCF!I61*DCF!H5</f>
-        <v>18030600000</v>
+        <v>18144000000</v>
       </c>
       <c r="D18" s="149"/>
       <c r="E18" s="150">
         <f>C18/(C18+C19)</f>
-        <v>0.84848402265397793</v>
+        <v>0.84928827730012568</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
@@ -11533,7 +11757,7 @@
       <c r="D19" s="151"/>
       <c r="E19" s="150">
         <f>C19/(C19+C18)</f>
-        <v>0.1515159773460221</v>
+        <v>0.15071172269987429</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
@@ -11544,7 +11768,7 @@
       <c r="D21" s="134"/>
       <c r="E21" s="153">
         <f>E18*C13+E19*C8</f>
-        <v>0.19090075624985225</v>
+        <v>0.19099252845010467</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
@@ -11574,4 +11798,861 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCBA2528-4CE8-4DC6-9EAF-7D5BAEA9729B}">
+  <dimension ref="B1:H74"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2" style="5" customWidth="1"/>
+    <col min="2" max="2" width="38" style="5" customWidth="1"/>
+    <col min="3" max="6" width="16" style="5" customWidth="1"/>
+    <col min="7" max="7" width="2" style="5" customWidth="1"/>
+    <col min="8" max="8" width="46" style="5" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" s="281" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="279" t="s">
+        <v>259</v>
+      </c>
+      <c r="C2" s="280"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="282"/>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="44" t="s">
+        <v>260</v>
+      </c>
+      <c r="C4" s="299">
+        <f>DCF!D7</f>
+        <v>46210</v>
+      </c>
+      <c r="H4" s="282"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="284" t="s">
+        <v>261</v>
+      </c>
+      <c r="C6" s="285"/>
+      <c r="D6" s="285"/>
+      <c r="E6" s="285"/>
+      <c r="F6" s="285"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="283" t="s">
+        <v>248</v>
+      </c>
+      <c r="D7" s="283" t="s">
+        <v>309</v>
+      </c>
+      <c r="E7" s="283" t="s">
+        <v>308</v>
+      </c>
+      <c r="F7" s="283" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="C8" s="298" t="s">
+        <v>306</v>
+      </c>
+      <c r="D8" s="298" t="s">
+        <v>263</v>
+      </c>
+      <c r="E8" s="298" t="s">
+        <v>307</v>
+      </c>
+      <c r="F8" s="298" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="34" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" s="283" t="s">
+        <v>266</v>
+      </c>
+      <c r="D9" s="283" t="s">
+        <v>266</v>
+      </c>
+      <c r="E9" s="283" t="s">
+        <v>266</v>
+      </c>
+      <c r="F9" s="283" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="C10" s="299">
+        <v>46387</v>
+      </c>
+      <c r="D10" s="299">
+        <v>46387</v>
+      </c>
+      <c r="E10" s="299">
+        <v>46203</v>
+      </c>
+      <c r="F10" s="299">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="34" t="s">
+        <v>268</v>
+      </c>
+      <c r="C11" s="286">
+        <f>FSM!D7</f>
+        <v>16</v>
+      </c>
+      <c r="D11" s="287">
+        <v>35.69</v>
+      </c>
+      <c r="E11" s="287">
+        <v>12.66</v>
+      </c>
+      <c r="F11" s="287">
+        <v>69.72</v>
+      </c>
+      <c r="H11" s="282"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="282" t="s">
+        <v>269</v>
+      </c>
+      <c r="C12" s="300">
+        <v>46210</v>
+      </c>
+      <c r="D12" s="300">
+        <v>46210</v>
+      </c>
+      <c r="E12" s="300">
+        <v>46210</v>
+      </c>
+      <c r="F12" s="300">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="284" t="s">
+        <v>314</v>
+      </c>
+      <c r="C14" s="285"/>
+      <c r="D14" s="285"/>
+      <c r="E14" s="285"/>
+      <c r="F14" s="285"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="34" t="s">
+        <v>270</v>
+      </c>
+      <c r="C15" s="289">
+        <f>DCF!I56</f>
+        <v>1134000000</v>
+      </c>
+      <c r="D15" s="290">
+        <v>2868140263</v>
+      </c>
+      <c r="E15" s="290">
+        <v>1986578999</v>
+      </c>
+      <c r="F15" s="290">
+        <v>1261875720</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="34" t="s">
+        <v>271</v>
+      </c>
+      <c r="C16" s="290">
+        <v>0</v>
+      </c>
+      <c r="D16" s="290">
+        <v>0</v>
+      </c>
+      <c r="E16" s="290">
+        <v>0</v>
+      </c>
+      <c r="F16" s="290">
+        <v>0</v>
+      </c>
+      <c r="H16" s="282"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="44" t="s">
+        <v>272</v>
+      </c>
+      <c r="C17" s="291">
+        <f>+C15+C16</f>
+        <v>1134000000</v>
+      </c>
+      <c r="D17" s="291">
+        <f>+D15+D16</f>
+        <v>2868140263</v>
+      </c>
+      <c r="E17" s="291">
+        <f>+E15+E16</f>
+        <v>1986578999</v>
+      </c>
+      <c r="F17" s="291">
+        <f>+F15+F16</f>
+        <v>1261875720</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="284" t="s">
+        <v>273</v>
+      </c>
+      <c r="C19" s="285"/>
+      <c r="D19" s="285"/>
+      <c r="E19" s="285"/>
+      <c r="F19" s="285"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="34" t="s">
+        <v>274</v>
+      </c>
+      <c r="C20" s="289">
+        <f>SUM(DCF!C57:C60)</f>
+        <v>3219770683</v>
+      </c>
+      <c r="D20" s="290">
+        <v>842054693</v>
+      </c>
+      <c r="E20" s="290">
+        <v>1217742500</v>
+      </c>
+      <c r="F20" s="290">
+        <v>149970052</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="C21" s="290"/>
+      <c r="D21" s="290"/>
+      <c r="E21" s="290"/>
+      <c r="F21" s="290"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="C22" s="289">
+        <f>SUM(DCF!C62:C64)</f>
+        <v>5594286609</v>
+      </c>
+      <c r="D22" s="290">
+        <v>16941003996</v>
+      </c>
+      <c r="E22" s="290">
+        <v>3273355000</v>
+      </c>
+      <c r="F22" s="290">
+        <v>38831683997</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="44" t="s">
+        <v>277</v>
+      </c>
+      <c r="C23" s="291">
+        <f>C20-C22</f>
+        <v>-2374515926</v>
+      </c>
+      <c r="D23" s="291">
+        <f t="shared" ref="D23:F23" si="0">SUM(D20:D21)-SUM(D22)</f>
+        <v>-16098949303</v>
+      </c>
+      <c r="E23" s="291">
+        <f t="shared" si="0"/>
+        <v>-2055612500</v>
+      </c>
+      <c r="F23" s="291">
+        <f t="shared" si="0"/>
+        <v>-38681713945</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="284" t="s">
+        <v>278</v>
+      </c>
+      <c r="C25" s="285"/>
+      <c r="D25" s="285"/>
+      <c r="E25" s="285"/>
+      <c r="F25" s="285"/>
+    </row>
+    <row r="26" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="44" t="s">
+        <v>279</v>
+      </c>
+      <c r="C26" s="291">
+        <f>C11*C17</f>
+        <v>18144000000</v>
+      </c>
+      <c r="D26" s="291">
+        <f t="shared" ref="D26:F26" si="1">D17*D11</f>
+        <v>102363925986.46999</v>
+      </c>
+      <c r="E26" s="291">
+        <f t="shared" si="1"/>
+        <v>25150090127.34</v>
+      </c>
+      <c r="F26" s="291">
+        <f t="shared" si="1"/>
+        <v>87977975198.399994</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="44" t="s">
+        <v>280</v>
+      </c>
+      <c r="C27" s="292">
+        <f>C26+C23</f>
+        <v>15769484074</v>
+      </c>
+      <c r="D27" s="292">
+        <f t="shared" ref="D27:F27" si="2">D26+D23</f>
+        <v>86264976683.469986</v>
+      </c>
+      <c r="E27" s="292">
+        <f t="shared" si="2"/>
+        <v>23094477627.34</v>
+      </c>
+      <c r="F27" s="292">
+        <f t="shared" si="2"/>
+        <v>49296261253.399994</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="284" t="s">
+        <v>281</v>
+      </c>
+      <c r="C29" s="285"/>
+      <c r="D29" s="285"/>
+      <c r="E29" s="285"/>
+      <c r="F29" s="285"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="282" t="s">
+        <v>282</v>
+      </c>
+      <c r="C30" s="288" t="s">
+        <v>283</v>
+      </c>
+      <c r="D30" s="288" t="s">
+        <v>283</v>
+      </c>
+      <c r="E30" s="288" t="s">
+        <v>283</v>
+      </c>
+      <c r="F30" s="288" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="289">
+        <f>FSM!F16</f>
+        <v>14412587014</v>
+      </c>
+      <c r="D31" s="290">
+        <v>26844075576</v>
+      </c>
+      <c r="E31" s="290">
+        <v>8602606000</v>
+      </c>
+      <c r="F31" s="290">
+        <v>22915657021</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="289">
+        <f>FSM!F35</f>
+        <v>660627360</v>
+      </c>
+      <c r="D32" s="290">
+        <v>15279059550</v>
+      </c>
+      <c r="E32" s="290">
+        <v>2541858400</v>
+      </c>
+      <c r="F32" s="290">
+        <v>8316306389</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="289">
+        <f>FSM!F24</f>
+        <v>580753378</v>
+      </c>
+      <c r="D33" s="290">
+        <v>12960330520</v>
+      </c>
+      <c r="E33" s="290">
+        <v>1798948000</v>
+      </c>
+      <c r="F33" s="290">
+        <v>8162886025</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="C34" s="289">
+        <f>FSM!F33</f>
+        <v>1138395311</v>
+      </c>
+      <c r="D34" s="290">
+        <v>11296540287</v>
+      </c>
+      <c r="E34" s="290">
+        <v>986964000</v>
+      </c>
+      <c r="F34" s="290">
+        <v>9352763248</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="282" t="s">
+        <v>284</v>
+      </c>
+      <c r="C35" s="293">
+        <f>+C32/C31</f>
+        <v>4.5836834106068834E-2</v>
+      </c>
+      <c r="D35" s="293">
+        <f>+D32/D31</f>
+        <v>0.56917808574716855</v>
+      </c>
+      <c r="E35" s="293">
+        <f>+E32/E31</f>
+        <v>0.29547539431655945</v>
+      </c>
+      <c r="F35" s="293">
+        <f>+F32/F31</f>
+        <v>0.36290935849576139</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B37" s="284" t="s">
+        <v>285</v>
+      </c>
+      <c r="C37" s="285"/>
+      <c r="D37" s="285"/>
+      <c r="E37" s="285"/>
+      <c r="F37" s="285"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="34" t="s">
+        <v>286</v>
+      </c>
+      <c r="C38" s="294">
+        <f>C27/C31</f>
+        <v>1.094146669066556</v>
+      </c>
+      <c r="D38" s="294">
+        <f t="shared" ref="D38:F38" si="3">D27/D31</f>
+        <v>3.213557361632351</v>
+      </c>
+      <c r="E38" s="294">
+        <f t="shared" si="3"/>
+        <v>2.6845908818025608</v>
+      </c>
+      <c r="F38" s="294">
+        <f t="shared" si="3"/>
+        <v>2.1512043581479992</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="44" t="s">
+        <v>287</v>
+      </c>
+      <c r="C39" s="295">
+        <f>C27/C32</f>
+        <v>23.870467723286545</v>
+      </c>
+      <c r="D39" s="295">
+        <f t="shared" ref="D39:F39" si="4">D27/D32</f>
+        <v>5.64596115364116</v>
+      </c>
+      <c r="E39" s="295">
+        <f t="shared" si="4"/>
+        <v>9.0856664664483286</v>
+      </c>
+      <c r="F39" s="295">
+        <f t="shared" si="4"/>
+        <v>5.9276629488548291</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="34" t="s">
+        <v>288</v>
+      </c>
+      <c r="C40" s="294">
+        <f>C27/C33</f>
+        <v>27.15349522082332</v>
+      </c>
+      <c r="D40" s="294">
+        <f t="shared" ref="D40:F40" si="5">D27/D33</f>
+        <v>6.6560784503410941</v>
+      </c>
+      <c r="E40" s="294">
+        <f t="shared" si="5"/>
+        <v>12.837768310890587</v>
+      </c>
+      <c r="F40" s="294">
+        <f t="shared" si="5"/>
+        <v>6.0390725905547598</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B41" s="44" t="s">
+        <v>289</v>
+      </c>
+      <c r="C41" s="295">
+        <f>C26/C34</f>
+        <v>15.938224467967789</v>
+      </c>
+      <c r="D41" s="295">
+        <f t="shared" ref="D41:F41" si="6">D26/D34</f>
+        <v>9.0615288739570872</v>
+      </c>
+      <c r="E41" s="295">
+        <f t="shared" si="6"/>
+        <v>25.482277091504859</v>
+      </c>
+      <c r="F41" s="295">
+        <f t="shared" si="6"/>
+        <v>9.4066291282646599</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B43" s="284" t="s">
+        <v>290</v>
+      </c>
+      <c r="C43" s="285"/>
+      <c r="D43" s="285"/>
+      <c r="E43" s="285"/>
+      <c r="F43" s="285"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C44" s="44" t="s">
+        <v>291</v>
+      </c>
+      <c r="D44" s="44" t="s">
+        <v>292</v>
+      </c>
+      <c r="E44" s="44" t="s">
+        <v>293</v>
+      </c>
+      <c r="F44" s="44" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B45" s="34" t="s">
+        <v>295</v>
+      </c>
+      <c r="C45" s="294">
+        <f>AVERAGE(D38:F38)</f>
+        <v>2.6831175338609703</v>
+      </c>
+      <c r="D45" s="294">
+        <f>AVERAGE(D39:F39)</f>
+        <v>6.8864301896481059</v>
+      </c>
+      <c r="E45" s="294">
+        <f>AVERAGE(D40:F40)</f>
+        <v>8.5109731172621466</v>
+      </c>
+      <c r="F45" s="294">
+        <f>AVERAGE(D41:F41)</f>
+        <v>14.650145031242202</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B46" s="44" t="s">
+        <v>296</v>
+      </c>
+      <c r="C46" s="295">
+        <f>MEDIAN(D38:F38)</f>
+        <v>2.6845908818025608</v>
+      </c>
+      <c r="D46" s="295">
+        <f>MEDIAN(D39:F39)</f>
+        <v>5.9276629488548291</v>
+      </c>
+      <c r="E46" s="295">
+        <f>MEDIAN(D40:F40)</f>
+        <v>6.6560784503410941</v>
+      </c>
+      <c r="F46" s="295">
+        <f>MEDIAN(D41:F41)</f>
+        <v>9.4066291282646599</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B47" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="C47" s="294">
+        <f>MAX(D38:F38)</f>
+        <v>3.213557361632351</v>
+      </c>
+      <c r="D47" s="294">
+        <f>MAX(D39:F39)</f>
+        <v>9.0856664664483286</v>
+      </c>
+      <c r="E47" s="294">
+        <f>MAX(D40:F40)</f>
+        <v>12.837768310890587</v>
+      </c>
+      <c r="F47" s="294">
+        <f>MAX(D41:F41)</f>
+        <v>25.482277091504859</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B48" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="C48" s="294">
+        <f>MIN(D38:F38)</f>
+        <v>2.1512043581479992</v>
+      </c>
+      <c r="D48" s="294">
+        <f>MIN(D39:F39)</f>
+        <v>5.64596115364116</v>
+      </c>
+      <c r="E48" s="294">
+        <f>MIN(D40:F40)</f>
+        <v>6.0390725905547598</v>
+      </c>
+      <c r="F48" s="294">
+        <f>MIN(D41:F41)</f>
+        <v>9.0615288739570872</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B50" s="284" t="s">
+        <v>312</v>
+      </c>
+      <c r="C50" s="285"/>
+      <c r="D50" s="285"/>
+      <c r="E50" s="285"/>
+      <c r="F50" s="285"/>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B51" s="44" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B52" s="34" t="s">
+        <v>298</v>
+      </c>
+      <c r="C52" s="294">
+        <f>D46</f>
+        <v>5.9276629488548291</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B53" s="34" t="s">
+        <v>299</v>
+      </c>
+      <c r="C53" s="296">
+        <f>C32</f>
+        <v>660627360</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B54" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="C54" s="296">
+        <f>C52*C53</f>
+        <v>3915976324.8717809</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B55" s="34" t="s">
+        <v>301</v>
+      </c>
+      <c r="C55" s="296">
+        <f>C23</f>
+        <v>-2374515926</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B56" s="34" t="s">
+        <v>302</v>
+      </c>
+      <c r="C56" s="296">
+        <f>C54-C55</f>
+        <v>6290492250.8717804</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="C57" s="296">
+        <f>$C$17</f>
+        <v>1134000000</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="44" t="s">
+        <v>303</v>
+      </c>
+      <c r="C58" s="297">
+        <f>C56/C57</f>
+        <v>5.547171297065062</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B60" s="44" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B61" s="34" t="s">
+        <v>305</v>
+      </c>
+      <c r="C61" s="294">
+        <f>F46</f>
+        <v>9.4066291282646599</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B62" s="34" t="s">
+        <v>313</v>
+      </c>
+      <c r="C62" s="296">
+        <f>C34</f>
+        <v>1138395311</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B63" s="34" t="s">
+        <v>302</v>
+      </c>
+      <c r="C63" s="296">
+        <f>C62*C61</f>
+        <v>10708462491.932507</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="C64" s="296">
+        <f>$C$17</f>
+        <v>1134000000</v>
+      </c>
+    </row>
+    <row r="65" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="44" t="s">
+        <v>303</v>
+      </c>
+      <c r="C65" s="297">
+        <f>C63/C64</f>
+        <v>9.4430886172244328</v>
+      </c>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B67" s="44" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B68" s="34" t="s">
+        <v>292</v>
+      </c>
+      <c r="C68" s="294">
+        <f>E46</f>
+        <v>6.6560784503410941</v>
+      </c>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B69" s="34" t="s">
+        <v>299</v>
+      </c>
+      <c r="C69" s="18">
+        <f>C32</f>
+        <v>660627360</v>
+      </c>
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B70" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="C70" s="18">
+        <f>C68*C69</f>
+        <v>4397187534.6017284</v>
+      </c>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B71" s="34" t="s">
+        <v>301</v>
+      </c>
+      <c r="C71" s="18">
+        <f>C55</f>
+        <v>-2374515926</v>
+      </c>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B72" s="34" t="s">
+        <v>302</v>
+      </c>
+      <c r="C72" s="18">
+        <f>C70-C71</f>
+        <v>6771703460.6017284</v>
+      </c>
+    </row>
+    <row r="73" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B73" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="C73" s="296">
+        <f>$C$17</f>
+        <v>1134000000</v>
+      </c>
+    </row>
+    <row r="74" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="44" t="s">
+        <v>303</v>
+      </c>
+      <c r="C74" s="297">
+        <f>C72/C73</f>
+        <v>5.9715198065270974</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>